<commit_message>
New Update from MarsCloud
</commit_message>
<xml_diff>
--- a/Target Folder/QA-Files/zh-CN/Continents of the World.xlsx
+++ b/Target Folder/QA-Files/zh-CN/Continents of the World.xlsx
@@ -13,7 +13,7 @@
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{D8162458-12AF-44B7-B9DE-111E538A2364}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="工作表1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -29,91 +29,91 @@
   <si>
     <r>
       <rPr/>
-      <t>The Continents of the World:A Comprehensive Overview</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>The Earth, our home, is a vast and diverse planet, teeming with life and natural wonders.One of the most fascinating aspects of our world is its division into continents—large, continuous landmasses that are separated by oceans.These continents are not only geographical entities but also cultural, historical, and ecological hubs that have shaped human civilization and the natural world.In this article, we will explore the seven continents of the world:Asia, Africa, North America, South America, Antarctica, Europe, and Australia.Each continent has its unique characteristics, from towering mountain ranges and sprawling deserts to dense forests and vibrant cultures.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>1. Asia:The Largest and Most Populous Continent</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>Asia is the largest continent on Earth, covering approximately 30% of the planet's land area.It is also the most populous, home to over 4.6 billion people, which is about 60% of the world's population.Asia is a continent of extremes, boasting the highest point on Earth—Mount Everest at 8,848 meters (29,029 feet)—and the lowest point, the Dead Sea, which lies at 430 meters (1,412 feet) below sea level.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>The continent is incredibly diverse, both geographically and culturally.It spans from the frozen tundras of Siberia to the tropical rainforests of Southeast Asia.Asia is also home to some of the world's oldest civilizations, including those in China, India, and Mesopotamia.Today, it is a dynamic region with rapidly growing economies, such as China, India, and Japan, which play a significant role in global affairs.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>Asia's cultural diversity is reflected in its languages, religions, and traditions.The continent is the birthplace of major world religions, including Hinduism, Buddhism, Islam, and Christianity.From the bustling streets of Tokyo to the serene temples of Bhutan, Asia offers a rich tapestry of experiences that continue to captivate travellers and scholars alike.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>2. Africa:The Cradle of Humanity</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>Africa is the second-largest continent, covering about 20% of the Earth's land area.It is often referred to as the "Cradle of Humanity" because it is widely believed that the first humans evolved their millions of years ago.Africa is a continent of immense natural beauty, with landscapes ranging from the Sahara Desert, the largest hot desert in the world, to the lush rainforests of the Congo Basin.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>The continent is home to 54 countries and over 1.3 billion people, making it one of the most culturally diverse regions on the planet.Africa is known for its rich history, with ancient civilizations such as Egypt, Mali, and Axum leaving behind a legacy of monumental architecture, art, and literature.The Great Pyramid of Giza, the Sphinx, and the rock-hewn churches of Lalibela are just a few examples of Africa's historical treasures.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>Africa is also a continent of contrasts.While it is rich in natural resources, including oil, diamonds, and gold, many African nations face challenges such as poverty, political instability, and health crises.However, the continent is also experiencing rapid economic growth and development, with countries like Nigeria, South Africa, and Kenya emerging as key players in the global economy.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>3. North America:A Land of Opportunity</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>North America is the third-largest continent, spanning from the Arctic Circle in the north to the tropical regions of Central America and the Caribbean in the south.It is home to 23 countries, including the United States, Canada, and Mexico, as well as numerous territories and dependencies.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>The continent is known for its diverse landscapes, which include the Rocky Mountains, the Great Plains, the Mississippi River, and the Grand Canyon.North America is also home to some of the world's most iconic cities, such as New York, Los Angeles, and Toronto, which are centers of culture, finance, and innovation.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>North America has a rich history, shaped by indigenous peoples, European colonization, and the African diaspora.The continent is a melting pot of cultures, with influences from Native American, European, African, and Asian traditions.这种文化多样性体现在非洲大陆的美食、音乐和艺术中。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>从经济角度来看，北美是世界上最繁荣的地区之一。美国和加拿大是世界上最大的经济体之一，拥有高度发达的基础设施、教育系统和医疗保健。然而，北美大陆也面临挑战，包括收入不平等、环境退化和政治两极分化。</t>
+      <t>世界各大洲：综合概述</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>地球，我们的家园，是一个广阔而多样的星球，生命和自然奇观在此繁衍生息。我们世界最迷人的方面之一是它被划分为各大洲——被海洋隔开的巨大连续陆块。这些大陆不仅是地理实体，也是文化、历史和生态中心，塑造了人类文明和自然世界。在本文中，我们将探讨世界七大洲：亚洲、非洲、北美洲、南美洲、南极洲、欧洲和澳大利亚。每个大陆都有其独特的特征，从高耸的山脉和广阔的沙漠到茂密的森林和充满活力的文化。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>1. 亚洲：面积最大、人口最多的大洲</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>亚洲是地球上最大的大陆，约占地球陆地面积的30%。它也是人口最多的大陆，拥有超过46亿人口，约占世界人口的60%。亚洲是一个充满极端的大陆，拥有地球上的最高点——珠穆朗玛峰，海拔8848米（29029英尺），以及最低点——死海，位于海平面以下430米（1412英尺）。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>该大陆在地理和文化上都极其多样化。它横跨西伯利亚的冰冻苔原到东南亚的热带雨林。亚洲也是世界上一些最古老文明的发源地，包括中国、印度和美索不达米亚的文明。如今，它是一个充满活力的地区，经济快速增长，如中国、印度和日本，在全球事务中发挥着重要作用。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>亚洲的文化多样性体现在其语言、宗教和传统中。该大陆是世界主要宗教的发源地，包括印度教、佛教、伊斯兰教和基督教。从东京熙熙攘攘的街道到不丹宁静的寺庙，亚洲提供了丰富的体验，继续吸引着旅行者和学者。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>2. 非洲：人类的摇篮</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>非洲是第二大洲，约占地球陆地面积的20%。它常被称为“人类的摇篮”，因为人们普遍认为第一批人类是在数百万年前在那里进化的。非洲是一个拥有巨大自然美景的大陆，其景观范围从世界上最大的热沙漠撒哈拉沙漠到刚果盆地茂盛的热带雨林。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>该大陆拥有54个国家和超过13亿人口，使其成为地球上文化最多样化的地区之一。非洲以其丰富的历史而闻名，古老的文明如埃及、马里和阿克苏姆留下了不朽的建筑、艺术和文学遗产。吉萨大金字塔、狮身人面像和拉利贝拉的岩石教堂只是非洲历史宝藏的几个例子。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>非洲也是一个充满对比的大陆。尽管它拥有丰富的自然资源，包括石油、钻石和黄金，但许多非洲国家面临贫困、政治不稳定和健康危机等挑战。然而，该大陆也正在经历快速的经济增长和发展，尼日利亚、南非和肯尼亚等国家正在成为全球经济中的关键参与者。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>3. 北美洲：机遇之地</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>北美洲是第三大洲，从北部的北极圈一直延伸到中美洲和加勒比海的热带地区。它拥有23个国家，包括美国、加拿大和墨西哥，以及众多领土和属地。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>该大陆以其多样的景观而闻名，其中包括落基山脉、大平原、密西西比河和大峡谷。北美洲也是世界上一些最具标志性城市的所在地，如纽约、洛杉矶和多伦多，它们是文化、金融和创新的中心。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>北美洲拥有丰富的历史，由原住民、欧洲殖民和非洲侨民塑造。该大陆是文化的熔炉，融合了美洲原住民、欧洲、非洲和亚洲的传统。这种文化多样性体现在非洲大陆的美食、音乐和艺术中。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>在经济上，北美洲是世界上最繁荣的地区之一。美国和加拿大是世界上最大的经济体之一，拥有高度发达的基础设施、教育系统和医疗保健。然而，北美洲也面临挑战，包括收入不平等、环境退化和政治两极分化。</t>
     </r>
   </si>
   <si>
@@ -125,25 +125,25 @@
   <si>
     <r>
       <rPr/>
-      <t>南美洲是第四大洲，以其令人惊叹的自然美景和丰富的文化遗产而闻名。它是巴西、阿根廷和哥伦比亚等12个国家的所在地，也是世界上最大的热带雨林——亚马逊雨林的所在地。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>这片大陆的特点是其多样的景观，包括安第斯山脉、阿塔卡马沙漠和潘塔纳尔湿地。南美洲也是世界上一些最具标志性地标的所在地，例如马丘比丘、基督救世主雕像和伊瓜苏瀑布。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>南美洲拥有丰富的文化历史，受到印加、玛雅和阿兹特克等土著文明以及欧洲殖民和非洲侨民的影响。这片大陆以其充满活力的音乐和舞蹈传统而闻名，包括桑巴、探戈和萨尔萨，以及其丰富多彩的节日，例如巴西狂欢节。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>从经济角度来看，南美洲是一个充满对比的地区。虽然巴西和阿根廷等国家拥有庞大且多样化的经济，但委内瑞拉等其他国家则面临重大的经济挑战。这片大陆还拥有丰富的自然资源，包括石油、铜和大豆，这些资源在全球经济中发挥着关键作用。</t>
+      <t>南美洲是第四大洲，以其令人惊叹的自然美景和丰富的文化遗产而闻名。它是12个国家的所在地，包括巴西、阿根廷和哥伦比亚，以及世界上最大的热带雨林亚马逊雨林。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>该大陆的特点是其多样的地貌，包括安第斯山脉、阿塔卡马沙漠和潘塔纳尔湿地。南美洲也是世界上一些最具标志性地标的所在地，例如马丘比丘、基督救世主雕像和伊瓜苏瀑布。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>南美洲拥有丰富的文化历史，由印加、玛雅和阿兹特克等原住民文明以及欧洲殖民和非洲侨民塑造。该大陆以其充满活力的音乐和舞蹈传统而闻名，包括桑巴、探戈和萨尔萨，以及其丰富多彩的节日，例如巴西的狂欢节。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>在经济上，南美洲是一个充满对比的地区。虽然巴西和阿根廷等国家拥有庞大且多元化的经济，但委内瑞拉等其他国家则面临重大的经济挑战。该大陆还拥有丰富的自然资源，包括石油、铜和大豆，这些资源在全球经济中发挥着关键作用。</t>
     </r>
   </si>
   <si>
@@ -155,19 +155,19 @@
   <si>
     <r>
       <rPr/>
-      <t>南极洲是第五大洲，也是地球上最偏远、最不适宜居住的地方。它是唯一没有土著人口的大陆，被一层厚厚的冰盖覆盖，其中含有世界上约70%的淡水。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>南极洲是一个极端的大陆，气温可低至-89.2°C（-128.6°F），风速可达320公里/小时（200英里/小时）以上。尽管条件恶劣，南极洲仍拥有独特的生态系统，包括企鹅、海豹和鲸鱼，以及各种在冰冷环境中繁衍的微生物。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>这片大陆受南极条约体系管辖，该体系将南极洲指定为科学保护区并禁止军事活动。来自不同国家的研究站对气候变化、地质学和天文学进行科学研究，使南极洲成为了解地球过去、现在和未来的重要地点。</t>
+      <t>南极洲是第五大洲，也是地球上最偏远和最不适宜居住的地方。它是唯一没有原住民的洲，被一层厚厚的冰盖覆盖，其中含有世界上约70%的淡水。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>南极洲是一个极端的大陆，气温可低至-89.2°C (-128.6°F)，风速可达320公里/小时 (200英里/小时) 以上。尽管条件恶劣，南极洲仍拥有独特的生态系统，包括企鹅、海豹和鲸鱼，以及各种在冰冷环境中 thriving 的微生物。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>该大陆受《南极条约体系》管辖，该体系将南极洲指定为科学保护区并禁止军事活动。来自不同国家的研究站对气候变化、地质学和天文学进行科学研究，使南极洲成为了解地球过去、现在和未来的重要地点。</t>
     </r>
   </si>
   <si>
@@ -179,49 +179,49 @@
   <si>
     <r>
       <rPr/>
-      <t>欧洲是第六大洲，但它是世界上人口最稠密、文化影响力最大的地区之一。它拥有44个国家，包括德国、法国和英国等主要强国，以及冰岛和马耳他等小国。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>欧洲以其丰富的历史而闻名，这段历史塑造了世界事件的进程。这片大陆是西方文明的诞生地，古希腊和罗马为现代哲学、法律和治理奠定了基础。欧洲也曾是重大历史事件的中心，包括文艺复兴、工业革命和两次世界大战。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>这片大陆的特点是其多样的景观，包括阿尔卑斯山、斯堪的纳维亚峡湾和地中海沿岸。欧洲也是世界上一些最具标志性城市的所在地，例如巴黎、伦敦和罗马，这些城市以其建筑、艺术和文化而闻名。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>从经济角度来看，欧洲是世界上最繁荣的地区之一，拥有高度发达的基础设施和高标准的生活水平。欧盟是一个由27个成员国组成的政治经济联盟，在全球事务中发挥着关键作用，并促进其成员国之间的合作和一体化。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>7. 澳大利亚：南半球的土地</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>澳大利亚是最小的大陆，也是唯一一个同时也是国家的国家。它位于南半球，被印度洋和太平洋环绕。澳大利亚以其独特的野生动物而闻名，包括袋鼠、考拉和鸭嘴兽，以及其令人惊叹的自然景观，例如大堡礁、乌鲁鲁和内陆地区。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>这片大陆拥有丰富的土著历史，原住民和托雷斯海峡岛民已在这片土地上生活了65,000多年。欧洲殖民始于18世纪末，如今，澳大利亚是一个拥有多元人口的多元文化社会。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>澳大利亚是一个高度发达的国家，经济实力雄厚，由采矿、农业和旅游业等产业驱动。该国以其高标准的生活、卓越的医疗和教育系统以及悉尼、墨尔本和布里斯班等充满活力的城市而闻名。</t>
+      <t>欧洲是第六大洲，但它是世界上人口最稠密、文化影响力最大的地区之一。它是44个国家的所在地，包括德国、法国和英国等主要大国，以及冰岛和马耳他等小国。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>欧洲以其丰富的历史而闻名，这段历史塑造了世界事件的进程。该大陆是西方文明的诞生地，古希腊和古罗马为现代哲学、法律和治理奠定了基础。欧洲也曾是重大历史事件的中心，包括文艺复兴、工业革命和两次世界大战。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>该大陆的特点是其多样的地貌，包括阿尔卑斯山、斯堪的纳维亚峡湾和地中海沿岸。欧洲也是世界上一些最具标志性城市的所在地，例如巴黎、伦敦和罗马，它们以其建筑、艺术和文化而闻名。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>在经济上，欧洲是世界上最繁荣的地区之一，拥有高度发达的基础设施和高标准的生活水平。欧盟是一个由27个成员国组成的政治经济联盟，在全球事务中发挥着关键作用，并促进其成员之间的合作和融合。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>7. 澳大利亚：“下澳”之地</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>澳大利亚是最小的大陆，也是唯一一个同时是国家的。它位于南半球，被印度洋和太平洋环绕。澳大利亚以其独特的野生动物而闻名，包括袋鼠、考拉和鸭嘴兽，以及其令人惊叹的自然景观，如大堡礁、乌鲁鲁和内陆地区。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>该大陆拥有丰富的原住民历史，澳大利亚原住民和托雷斯海峡岛民已在这片土地上生活了65,000多年。欧洲殖民始于18世纪末，如今，澳大利亚是一个拥有多元人口的多元文化社会。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>澳大利亚是一个高度发达的国家，经济实力雄厚，由采矿、农业和旅游等产业驱动。该国以其高标准的生活水平、卓越的医疗保健和教育系统以及悉尼、墨尔本和布里斯班等充满活力的城市而闻名。</t>
     </r>
   </si>
   <si>
@@ -233,13 +233,13 @@
   <si>
     <r>
       <rPr/>
-      <t>世界各大洲不仅仅是地理划分；它们是人类文明和自然世界的基础。每个大陆都有其独特的特征，从亚洲高耸的山峰到南极洲冰冻的荒野。它们共同构成了一个复杂而相互关联的系统，维持着地球上的生命。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>随着我们不断探索和了解各大洲，我们对地球的多样性和美丽有了更深刻的认识。无论是非洲丰富的文化遗产、北美洲的经济实力，还是南美洲的自然奇观，每个大陆都有其独特之处。通过了解和尊重这些差异，我们可以共同努力，为子孙后代创造一个更可持续、更和谐的世界。</t>
+      <t>世界各大洲不仅仅是地理上的划分；它们是人类文明和自然世界的基础。每个大陆都有其独特的特征，从亚洲高耸的山峰到南极洲冰冻的荒野。它们共同构成了一个复杂而相互关联的系统，维持着地球上的生命。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>随着我们继续探索和了解各大洲，我们对地球的多样性和美丽有了更深的认识。无论是非洲丰富的文化遗产、北美洲的经济实力，还是南美洲的自然奇观，每个大陆都有其独特之处。通过了解和尊重这些差异，我们可以共同努力，为子孙后代创造一个更可持续、更和谐的世界。</t>
     </r>
   </si>
   <si>
@@ -263,7 +263,7 @@
       <rPr>
         <family val="2"/>
       </rPr>
-      <t>：作为最大的大陆，亚洲对全球地理有着深远的影响。它是喜马拉雅山脉的所在地，喜马拉雅山脉影响着整个南亚及其他地区的天气模式。青藏高原常被称为“世界屋脊”，影响着季风系统，这对印度和孟加拉国等国家的农业至关重要。</t>
+      <t>：作为最大的大陆，亚洲对全球地理有着深远的影响。喜马拉雅山脉位于亚洲，影响着南亚及其他地区的天气模式。青藏高原常被称为“世界屋脊”，影响着季风系统，这对印度和孟加拉国等国家的农业至关重要。</t>
     </r>
   </si>
   <si>
@@ -287,7 +287,7 @@
       <rPr>
         <family val="2"/>
       </rPr>
-      <t>：落基山脉和大平原影响着天气模式，而密西西比河流域是世界上最肥沃的农业区之一。北美洲还拥有显著的生物多样性，从北极苔原到西南部的沙漠。</t>
+      <t>：落基山脉和大平原影响着天气模式，而密西西比河流域是世界上最肥沃的农业区之一。北美洲还拥有丰富的生物多样性，从北极苔原到西南部的沙漠。</t>
     </r>
   </si>
   <si>
@@ -311,7 +311,7 @@
       <rPr>
         <family val="2"/>
       </rPr>
-      <t>：南极冰盖含有全球约70%的淡水。由于气候变化导致的融化可能导致海平面上升，影响全球沿海城市。</t>
+      <t>：南极冰盖含有全球约70%的淡水。气候变化导致的融化可能导致海平面上升，影响全球沿海城市。</t>
     </r>
   </si>
   <si>
@@ -323,7 +323,7 @@
       <rPr>
         <family val="2"/>
       </rPr>
-      <t>：欧洲多样化的景观，从阿尔卑斯山到斯堪的纳维亚峡湾，影响着区域气候并支持着丰富的生态系统。该大陆的河流，如多瑙河和莱茵河，对交通和农业至关重要。</t>
+      <t>：欧洲多样化的景观，从阿尔卑斯山到斯堪的纳维亚峡湾，影响着区域气候并支持着丰富的生态系统。欧洲的河流，如多瑙河和莱茵河，对交通和农业至关重要。</t>
     </r>
   </si>
   <si>
@@ -335,7 +335,7 @@
       <rPr>
         <family val="2"/>
       </rPr>
-      <t>：澳大利亚独特的生态系统，包括大堡礁和内陆地区，对全球生物多样性做出了贡献。然而，它对气候变化的脆弱性，如丛林大火和珊瑚白化等事件所示，凸显了全球生态系统的相互关联性。</t>
+      <t>：澳大利亚独特的生态系统，包括大堡礁和内陆地区，为全球生物多样性做出了贡献。然而，其对气候变化的脆弱性，如森林大火和珊瑚白化等事件所示，凸显了全球生态系统的相互关联性。</t>
     </r>
   </si>
   <si>
@@ -353,7 +353,7 @@
       <rPr>
         <family val="2"/>
       </rPr>
-      <t>：作为主要宗教（印度教、佛教、伊斯兰教和基督教）的发源地，亚洲塑造了全球灵性和哲学。中国和印度等古代文明对科学、数学和文学做出了贡献，影响了世界数千年。</t>
+      <t>：作为主要宗教（印度教、佛教、伊斯兰教和基督教）的发源地，亚洲塑造了全球的灵性和哲学。中国和印度等古代文明对科学、数学和文学做出了贡献，影响了世界数千年。</t>
     </r>
   </si>
   <si>
@@ -365,7 +365,7 @@
       <rPr>
         <family val="2"/>
       </rPr>
-      <t>：非洲常被称为“人类摇篮”，是最初人类进化的地方。其丰富的文化遗产，从古埃及到马里帝国，在艺术、建筑和历史上留下了不可磨灭的印记。</t>
+      <t>：非洲常被称为“人类摇篮”，是最初人类的进化之地。其丰富的文化遗产，从古埃及到马里帝国，在艺术、建筑和历史上留下了不可磨灭的印记。</t>
     </r>
   </si>
   <si>
@@ -377,7 +377,7 @@
       <rPr>
         <family val="2"/>
       </rPr>
-      <t>：北美洲的土著文化，如纳瓦霍人和易洛魁人，为全球可持续发展和环境管理知识做出了贡献。欧洲殖民和跨大西洋奴隶贸易对全球人口和文化产生了持久影响。</t>
+      <t>：北美洲的土著文化，如纳瓦霍族和易洛魁族，为全球可持续发展和环境管理知识做出了贡献。欧洲殖民和跨大西洋奴隶贸易对全球人口结构和文化产生了持久影响。</t>
     </r>
   </si>
   <si>
@@ -389,7 +389,7 @@
       <rPr>
         <family val="2"/>
       </rPr>
-      <t>：印加、玛雅和阿兹特克文明留下了不朽的建筑和先进的农业实践。非洲大陆充满活力的文化，包括音乐、舞蹈和节日，影响了全球艺术和娱乐。</t>
+      <t>：印加、玛雅和阿兹特克文明留下了不朽的建筑和先进的农业实践。该大陆充满活力的文化，包括音乐、舞蹈和节日，影响了全球艺术和娱乐。</t>
     </r>
   </si>
   <si>
@@ -413,7 +413,7 @@
       <rPr>
         <family val="2"/>
       </rPr>
-      <t>：拥有超过 65,000 年历史的澳大利亚原住民文化，为可持续生活和与土地的联系提供了深刻的见解。澳大利亚的多元文化社会反映了其作为全球移民中心的地位。</t>
+      <t>：澳大利亚原住民文化拥有超过 65,000 年的历史，为可持续生活和与土地的联系提供了深刻的见解。澳大利亚的多元文化社会反映了其作为全球移民中心的地位。</t>
     </r>
   </si>
   <si>
@@ -431,7 +431,7 @@
       <rPr>
         <family val="2"/>
       </rPr>
-      <t>：亚洲是全球经济强国，中国、印度和日本等国家推动着国际贸易和创新。亚洲是电子产品、纺织品和汽车的主要生产国，影响着全球市场。</t>
+      <t>：亚洲是全球经济强国，中国、印度和日本等国家推动着国际贸易和创新。该大陆是电子产品、纺织品和汽车的主要生产商，影响着全球市场。</t>
     </r>
   </si>
   <si>
@@ -443,7 +443,7 @@
       <rPr>
         <family val="2"/>
       </rPr>
-      <t>：非洲拥有丰富的自然资源，包括石油、钻石和黄金，这些对全球经济至关重要。然而，贫困和不平等等经济挑战在许多地区依然存在。</t>
+      <t>：非洲拥有丰富的自然资源，包括石油、钻石和黄金，这些对全球经济至关重要。然而，贫困和不平等之类的经济挑战在许多地区依然存在。</t>
     </r>
   </si>
   <si>
@@ -455,7 +455,7 @@
       <rPr>
         <family val="2"/>
       </rPr>
-      <t>：美国和加拿大是世界上最大的经济体之一，对技术、金融和娱乐做出了重大贡献。北美洲的农业产出养活了全球数百万人口。</t>
+      <t>：美国和加拿大是世界上最大的经济体之一，对技术、金融和娱乐做出了重大贡献。北美洲的农业产出养活了全球数百万人。</t>
     </r>
   </si>
   <si>
@@ -467,7 +467,7 @@
       <rPr>
         <family val="2"/>
       </rPr>
-      <t>：南美洲是大豆、咖啡和铜等商品的主要出口国。巴西是南美洲最大的经济体，在全球贸易中发挥着关键作用。</t>
+      <t>：该大陆是大豆、咖啡和铜等商品的主要出口国。巴西是南美洲最大的经济体，在全球贸易中扮演着关键角色。</t>
     </r>
   </si>
   <si>
@@ -479,7 +479,7 @@
       <rPr>
         <family val="2"/>
       </rPr>
-      <t>：欧盟是世界上最大的经济集团之一，促进其成员国之间的贸易与合作。欧洲也是可再生能源和可持续发展的领导者。</t>
+      <t>：欧盟是世界上最大的经济集团之一，促进其成员国之间的贸易和合作。欧洲也是可再生能源和可持续发展的领导者。</t>
     </r>
   </si>
   <si>
@@ -509,7 +509,7 @@
       <rPr>
         <family val="2"/>
       </rPr>
-      <t>：亚洲的地缘政治意义不可否认，中国、印度和日本等国家在国际关系中发挥着关键作用。该地区的冲突和联盟塑造了全球政治。</t>
+      <t>：亚洲的地缘政治意义不可否认，中国、印度和日本等国家在国际关系中扮演着关键角色。该地区的冲突和联盟影响着全球政治。</t>
     </r>
   </si>
   <si>
@@ -521,7 +521,7 @@
       <rPr>
         <family val="2"/>
       </rPr>
-      <t>：非洲不断增长的人口和年轻的人口结构使其成为全球发展中的关键参与者。非洲大陆为应对贫困、健康危机和政治不稳定等挑战所做的努力具有深远影响。</t>
+      <t>：非洲不断增长的人口和年轻的人口结构使其成为全球发展中的关键参与者。该大陆应对贫困、健康危机和政治不稳定等挑战的努力具有深远的影响。</t>
     </r>
   </si>
   <si>
@@ -545,7 +545,7 @@
       <rPr>
         <family val="2"/>
       </rPr>
-      <t>：南美洲的政治格局，从委内瑞拉的社会主义运动到智利的民主转型，反映了其多元的意识形态和争取平等的斗争。</t>
+      <t>：该大陆的政治格局，从委内瑞拉的社会主义运动到智利的民主转型，反映了其多元的意识形态和对平等的斗争。</t>
     </r>
   </si>
   <si>
@@ -569,7 +569,7 @@
       <rPr>
         <family val="2"/>
       </rPr>
-      <t>：澳大利亚在亚太地区的作用以及其对国际援助和环境保护的承诺，凸显了其全球影响力。</t>
+      <t>：澳大利亚在亚太地区的作用及其对国际援助和环境保护的承诺突显了其全球影响力。</t>
     </r>
   </si>
   <si>
@@ -617,7 +617,7 @@
       <rPr>
         <family val="2"/>
       </rPr>
-      <t>：经历野火、飓风和北极冰融化。</t>
+      <t>：经历森林火灾、飓风和北极冰融化。</t>
     </r>
   </si>
   <si>
@@ -653,7 +653,7 @@
       <rPr>
         <family val="2"/>
       </rPr>
-      <t>：面临气候变化导致的酷热和洪水。</t>
+      <t>：面临气候变化导致的热浪和洪水。</t>
     </r>
   </si>
   <si>
@@ -677,7 +677,7 @@
   <si>
     <r>
       <rPr/>
-      <t>各大洲通过贸易、移民和技术相互关联。例如：</t>
+      <t>各大洲通过贸易、移民和技术相互连接。例如：</t>
     </r>
   </si>
   <si>
@@ -701,7 +701,7 @@
       <rPr>
         <family val="2"/>
       </rPr>
-      <t>：人们为了工作、教育和寻求庇护而在各大洲之间迁移，丰富了文化和经济。</t>
+      <t>：人们为了工作、教育和寻求庇护而在各大洲之间迁徙，丰富了文化和经济。</t>
     </r>
   </si>
   <si>
@@ -719,97 +719,97 @@
   <si>
     <r>
       <rPr/>
-      <t>世界各大洲并非孤立的实体，而是全球体系中相互关联的部分。它们在地理、文化、经济和政治方面的影响深刻地塑造着世界。面对气候变化、不平等和冲突等全球性挑战，了解各大洲的作用和贡献对于促进合作、为全人类创造可持续的未来至关重要。通过认识到各大洲的多样性和相互关联性，我们可以共同努力应对共同挑战，建设一个更美好的世界。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>The Continents of the World:A Comprehensive Overview</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>The Earth, our home, is a vast and diverse planet, teeming with life and natural wonders.One of the most fascinating aspects of our world is its division into continents—large, continuous landmasses that are separated by oceans.These continents are not only geographical entities but also cultural, historical, and ecological hubs that have shaped human civilization and the natural world.In this article, we will explore the seven continents of the world:Asia, Africa, North America, South America, Antarctica, Europe, and Australia.Each continent has its unique characteristics, from towering mountain ranges and sprawling deserts to dense forests and vibrant cultures.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>1. Asia:The Largest and Most Populous Continent</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>Asia is the largest continent on Earth, covering approximately 30% of the planet's land area.It is also the most populous, home to over 4.6 billion people, which is about 60% of the world's population.Asia is a continent of extremes, boasting the highest point on Earth—Mount Everest at 8,848 meters (29,029 feet)—and the lowest point, the Dead Sea, which lies at 430 meters (1,412 feet) below sea level.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>The continent is incredibly diverse, both geographically and culturally.It spans from the frozen tundras of Siberia to the tropical rainforests of Southeast Asia.Asia is also home to some of the world's oldest civilizations, including those in China, India, and Mesopotamia.Today, it is a dynamic region with rapidly growing economies, such as China, India, and Japan, which play a significant role in global affairs.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>Asia's cultural diversity is reflected in its languages, religions, and traditions.The continent is the birthplace of major world religions, including Hinduism, Buddhism, Islam, and Christianity.From the bustling streets of Tokyo to the serene temples of Bhutan, Asia offers a rich tapestry of experiences that continue to captivate travellers and scholars alike.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>2. Africa:The Cradle of Humanity</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>Africa is the second-largest continent, covering about 20% of the Earth's land area.It is often referred to as the "Cradle of Humanity" because it is widely believed that the first humans evolved their millions of years ago.Africa is a continent of immense natural beauty, with landscapes ranging from the Sahara Desert, the largest hot desert in the world, to the lush rainforests of the Congo Basin.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>The continent is home to 54 countries and over 1.3 billion people, making it one of the most culturally diverse regions on the planet.Africa is known for its rich history, with ancient civilizations such as Egypt, Mali, and Axum leaving behind a legacy of monumental architecture, art, and literature.The Great Pyramid of Giza, the Sphinx, and the rock-hewn churches of Lalibela are just a few examples of Africa's historical treasures.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>Africa is also a continent of contrasts.While it is rich in natural resources, including oil, diamonds, and gold, many African nations face challenges such as poverty, political instability, and health crises.However, the continent is also experiencing rapid economic growth and development, with countries like Nigeria, South Africa, and Kenya emerging as key players in the global economy.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>3. North America:A Land of Opportunity</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>North America is the third-largest continent, spanning from the Arctic Circle in the north to the tropical regions of Central America and the Caribbean in the south.It is home to 23 countries, including the United States, Canada, and Mexico, as well as numerous territories and dependencies.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>The continent is known for its diverse landscapes, which include the Rocky Mountains, the Great Plains, the Mississippi River, and the Grand Canyon.North America is also home to some of the world's most iconic cities, such as New York, Los Angeles, and Toronto, which are centers of culture, finance, and innovation.</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>North America has a rich history, shaped by indigenous peoples, European colonization, and the African diaspora.The continent is a melting pot of cultures, with influences from Native American, European, African, and Asian traditions.这种文化多样性体现在非洲大陆的美食、音乐和艺术中。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>从经济角度来看，北美是世界上最繁荣的地区之一。美国和加拿大是世界上最大的经济体之一，拥有高度发达的基础设施、教育系统和医疗保健。然而，北美大陆也面临挑战，包括收入不平等、环境退化和政治两极分化。</t>
+      <t>世界各大洲并非孤立的实体，而是全球系统中相互关联的部分。它们的地理、文化、经济和政治影响深刻地塑造着世界。当我们面临气候变化、不平等和冲突等全球性挑战时，了解每个大洲的作用和贡献对于促进合作、为所有人创造可持续的未来至关重要。通过认识到各大洲的多样性和相互关联性，我们可以共同努力应对共同挑战，建设一个更美好的世界。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>世界各大洲：综合概述</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>地球，我们的家园，是一个广阔而多样的星球，生命和自然奇观在此繁衍生息。我们世界最迷人的方面之一是它被划分为各大洲——被海洋隔开的巨大连续陆块。这些大陆不仅是地理实体，也是文化、历史和生态中心，塑造了人类文明和自然世界。在本文中，我们将探讨世界七大洲：亚洲、非洲、北美洲、南美洲、南极洲、欧洲和澳大利亚。每个大陆都有其独特的特征，从高耸的山脉和广阔的沙漠到茂密的森林和充满活力的文化。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>1. 亚洲：面积最大、人口最多的大洲</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>亚洲是地球上最大的大陆，约占地球陆地面积的30%。它也是人口最多的大陆，拥有超过46亿人口，约占世界人口的60%。亚洲是一个充满极端的大陆，拥有地球上的最高点——珠穆朗玛峰，海拔8848米（29029英尺），以及最低点——死海，位于海平面以下430米（1412英尺）。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>该大陆在地理和文化上都极其多样化。它横跨西伯利亚的冰冻苔原到东南亚的热带雨林。亚洲也是世界上一些最古老文明的发源地，包括中国、印度和美索不达米亚的文明。如今，它是一个充满活力的地区，经济快速增长，如中国、印度和日本，在全球事务中发挥着重要作用。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>亚洲的文化多样性体现在其语言、宗教和传统中。该大陆是世界主要宗教的发源地，包括印度教、佛教、伊斯兰教和基督教。从东京熙熙攘攘的街道到不丹宁静的寺庙，亚洲提供了丰富的体验，继续吸引着旅行者和学者。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>2. 非洲：人类的摇篮</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>非洲是第二大洲，约占地球陆地面积的20%。它常被称为“人类的摇篮”，因为人们普遍认为第一批人类是在数百万年前在那里进化的。非洲是一个拥有巨大自然美景的大陆，其景观范围从世界上最大的热沙漠撒哈拉沙漠到刚果盆地茂盛的热带雨林。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>该大陆拥有54个国家和超过13亿人口，使其成为地球上文化最多样化的地区之一。非洲以其丰富的历史而闻名，古老的文明如埃及、马里和阿克苏姆留下了不朽的建筑、艺术和文学遗产。吉萨大金字塔、狮身人面像和拉利贝拉的岩石教堂只是非洲历史宝藏的几个例子。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>非洲也是一个充满对比的大陆。尽管它拥有丰富的自然资源，包括石油、钻石和黄金，但许多非洲国家面临贫困、政治不稳定和健康危机等挑战。然而，该大陆也正在经历快速的经济增长和发展，尼日利亚、南非和肯尼亚等国家正在成为全球经济中的关键参与者。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>3. 北美洲：机遇之地</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>北美洲是第三大洲，从北部的北极圈一直延伸到中美洲和加勒比海的热带地区。它拥有23个国家，包括美国、加拿大和墨西哥，以及众多领土和属地。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>该大陆以其多样的景观而闻名，其中包括落基山脉、大平原、密西西比河和大峡谷。北美洲也是世界上一些最具标志性城市的所在地，如纽约、洛杉矶和多伦多，它们是文化、金融和创新的中心。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>北美洲拥有丰富的历史，由原住民、欧洲殖民和非洲侨民塑造。该大陆是文化的熔炉，融合了美洲原住民、欧洲、非洲和亚洲的传统。这种文化多样性体现在非洲大陆的美食、音乐和艺术中。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>在经济上，北美洲是世界上最繁荣的地区之一。美国和加拿大是世界上最大的经济体之一，拥有高度发达的基础设施、教育系统和医疗保健。然而，北美洲也面临挑战，包括收入不平等、环境退化和政治两极分化。</t>
     </r>
   </si>
   <si>
@@ -821,25 +821,25 @@
   <si>
     <r>
       <rPr/>
-      <t>南美洲是第四大洲，以其令人惊叹的自然美景和丰富的文化遗产而闻名。它是巴西、阿根廷和哥伦比亚等12个国家的所在地，也是世界上最大的热带雨林——亚马逊雨林的所在地。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>这片大陆的特点是其多样的景观，包括安第斯山脉、阿塔卡马沙漠和潘塔纳尔湿地。南美洲也是世界上一些最具标志性地标的所在地，例如马丘比丘、基督救世主雕像和伊瓜苏瀑布。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>南美洲拥有丰富的文化历史，受到印加、玛雅和阿兹特克等土著文明以及欧洲殖民和非洲侨民的影响。这片大陆以其充满活力的音乐和舞蹈传统而闻名，包括桑巴、探戈和萨尔萨，以及其丰富多彩的节日，例如巴西狂欢节。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>从经济角度来看，南美洲是一个充满对比的地区。虽然巴西和阿根廷等国家拥有庞大且多样化的经济，但委内瑞拉等其他国家则面临重大的经济挑战。这片大陆还拥有丰富的自然资源，包括石油、铜和大豆，这些资源在全球经济中发挥着关键作用。</t>
+      <t>南美洲是第四大洲，以其令人惊叹的自然美景和丰富的文化遗产而闻名。它是12个国家的所在地，包括巴西、阿根廷和哥伦比亚，以及世界上最大的热带雨林亚马逊雨林。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>该大陆的特点是其多样的地貌，包括安第斯山脉、阿塔卡马沙漠和潘塔纳尔湿地。南美洲也是世界上一些最具标志性地标的所在地，例如马丘比丘、基督救世主雕像和伊瓜苏瀑布。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>南美洲拥有丰富的文化历史，由印加、玛雅和阿兹特克等原住民文明以及欧洲殖民和非洲侨民塑造。该大陆以其充满活力的音乐和舞蹈传统而闻名，包括桑巴、探戈和萨尔萨，以及其丰富多彩的节日，例如巴西的狂欢节。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>在经济上，南美洲是一个充满对比的地区。虽然巴西和阿根廷等国家拥有庞大且多元化的经济，但委内瑞拉等其他国家则面临重大的经济挑战。该大陆还拥有丰富的自然资源，包括石油、铜和大豆，这些资源在全球经济中发挥着关键作用。</t>
     </r>
   </si>
   <si>
@@ -851,19 +851,19 @@
   <si>
     <r>
       <rPr/>
-      <t>南极洲是第五大洲，也是地球上最偏远、最不适宜居住的地方。它是唯一没有土著人口的大陆，被一层厚厚的冰盖覆盖，其中含有世界上约70%的淡水。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>南极洲是一个极端的大陆，气温可低至-89.2°C（-128.6°F），风速可达320公里/小时（200英里/小时）以上。尽管条件恶劣，南极洲仍拥有独特的生态系统，包括企鹅、海豹和鲸鱼，以及各种在冰冷环境中繁衍的微生物。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>这片大陆受南极条约体系管辖，该体系将南极洲指定为科学保护区并禁止军事活动。来自不同国家的研究站对气候变化、地质学和天文学进行科学研究，使南极洲成为了解地球过去、现在和未来的重要地点。</t>
+      <t>南极洲是第五大洲，也是地球上最偏远和最不适宜居住的地方。它是唯一没有原住民的洲，被一层厚厚的冰盖覆盖，其中含有世界上约70%的淡水。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>南极洲是一个极端的大陆，气温可低至-89.2°C (-128.6°F)，风速可达320公里/小时 (200英里/小时) 以上。尽管条件恶劣，南极洲仍拥有独特的生态系统，包括企鹅、海豹和鲸鱼，以及各种在冰冷环境中 thriving 的微生物。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>该大陆受《南极条约体系》管辖，该体系将南极洲指定为科学保护区并禁止军事活动。来自不同国家的研究站对气候变化、地质学和天文学进行科学研究，使南极洲成为了解地球过去、现在和未来的重要地点。</t>
     </r>
   </si>
   <si>
@@ -875,49 +875,49 @@
   <si>
     <r>
       <rPr/>
-      <t>欧洲是第六大洲，但它是世界上人口最稠密、文化影响力最大的地区之一。它拥有44个国家，包括德国、法国和英国等主要强国，以及冰岛和马耳他等小国。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>欧洲以其丰富的历史而闻名，这段历史塑造了世界事件的进程。这片大陆是西方文明的诞生地，古希腊和罗马为现代哲学、法律和治理奠定了基础。欧洲也曾是重大历史事件的中心，包括文艺复兴、工业革命和两次世界大战。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>这片大陆的特点是其多样的景观，包括阿尔卑斯山、斯堪的纳维亚峡湾和地中海沿岸。欧洲也是世界上一些最具标志性城市的所在地，例如巴黎、伦敦和罗马，这些城市以其建筑、艺术和文化而闻名。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>从经济角度来看，欧洲是世界上最繁荣的地区之一，拥有高度发达的基础设施和高标准的生活水平。欧盟是一个由27个成员国组成的政治经济联盟，在全球事务中发挥着关键作用，并促进其成员国之间的合作和一体化。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>7. 澳大利亚：南半球的土地</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>澳大利亚是最小的大陆，也是唯一一个同时也是国家的国家。它位于南半球，被印度洋和太平洋环绕。澳大利亚以其独特的野生动物而闻名，包括袋鼠、考拉和鸭嘴兽，以及其令人惊叹的自然景观，例如大堡礁、乌鲁鲁和内陆地区。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>这片大陆拥有丰富的土著历史，原住民和托雷斯海峡岛民已在这片土地上生活了65,000多年。欧洲殖民始于18世纪末，如今，澳大利亚是一个拥有多元人口的多元文化社会。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>澳大利亚是一个高度发达的国家，经济实力雄厚，由采矿、农业和旅游业等产业驱动。该国以其高标准的生活、卓越的医疗和教育系统以及悉尼、墨尔本和布里斯班等充满活力的城市而闻名。</t>
+      <t>欧洲是第六大洲，但它是世界上人口最稠密、文化影响力最大的地区之一。它是44个国家的所在地，包括德国、法国和英国等主要大国，以及冰岛和马耳他等小国。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>欧洲以其丰富的历史而闻名，这段历史塑造了世界事件的进程。该大陆是西方文明的诞生地，古希腊和古罗马为现代哲学、法律和治理奠定了基础。欧洲也曾是重大历史事件的中心，包括文艺复兴、工业革命和两次世界大战。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>该大陆的特点是其多样的地貌，包括阿尔卑斯山、斯堪的纳维亚峡湾和地中海沿岸。欧洲也是世界上一些最具标志性城市的所在地，例如巴黎、伦敦和罗马，它们以其建筑、艺术和文化而闻名。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>在经济上，欧洲是世界上最繁荣的地区之一，拥有高度发达的基础设施和高标准的生活水平。欧盟是一个由27个成员国组成的政治经济联盟，在全球事务中发挥着关键作用，并促进其成员之间的合作和融合。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>7. 澳大利亚：“下澳”之地</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>澳大利亚是最小的大陆，也是唯一一个同时是国家的。它位于南半球，被印度洋和太平洋环绕。澳大利亚以其独特的野生动物而闻名，包括袋鼠、考拉和鸭嘴兽，以及其令人惊叹的自然景观，如大堡礁、乌鲁鲁和内陆地区。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>该大陆拥有丰富的原住民历史，澳大利亚原住民和托雷斯海峡岛民已在这片土地上生活了65,000多年。欧洲殖民始于18世纪末，如今，澳大利亚是一个拥有多元人口的多元文化社会。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>澳大利亚是一个高度发达的国家，经济实力雄厚，由采矿、农业和旅游等产业驱动。该国以其高标准的生活水平、卓越的医疗保健和教育系统以及悉尼、墨尔本和布里斯班等充满活力的城市而闻名。</t>
     </r>
   </si>
   <si>
@@ -929,13 +929,13 @@
   <si>
     <r>
       <rPr/>
-      <t>世界各大洲不仅仅是地理划分；它们是人类文明和自然世界的基础。每个大陆都有其独特的特征，从亚洲高耸的山峰到南极洲冰冻的荒野。它们共同构成了一个复杂而相互关联的系统，维持着地球上的生命。</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr/>
-      <t>随着我们不断探索和了解各大洲，我们对地球的多样性和美丽有了更深刻的认识。无论是非洲丰富的文化遗产、北美洲的经济实力，还是南美洲的自然奇观，每个大陆都有其独特之处。通过了解和尊重这些差异，我们可以共同努力，为子孙后代创造一个更可持续、更和谐的世界。</t>
+      <t>世界各大洲不仅仅是地理上的划分；它们是人类文明和自然世界的基础。每个大陆都有其独特的特征，从亚洲高耸的山峰到南极洲冰冻的荒野。它们共同构成了一个复杂而相互关联的系统，维持着地球上的生命。</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr/>
+      <t>随着我们继续探索和了解各大洲，我们对地球的多样性和美丽有了更深的认识。无论是非洲丰富的文化遗产、北美洲的经济实力，还是南美洲的自然奇观，每个大陆都有其独特之处。通过了解和尊重这些差异，我们可以共同努力，为子孙后代创造一个更可持续、更和谐的世界。</t>
     </r>
   </si>
   <si>
@@ -959,7 +959,7 @@
       <rPr>
         <family val="2"/>
       </rPr>
-      <t>：作为最大的大陆，亚洲对全球地理有着深远的影响。它是喜马拉雅山脉的所在地，喜马拉雅山脉影响着整个南亚及其他地区的天气模式。青藏高原常被称为“世界屋脊”，影响着季风系统，这对印度和孟加拉国等国家的农业至关重要。</t>
+      <t>：作为最大的大陆，亚洲对全球地理有着深远的影响。喜马拉雅山脉位于亚洲，影响着南亚及其他地区的天气模式。青藏高原常被称为“世界屋脊”，影响着季风系统，这对印度和孟加拉国等国家的农业至关重要。</t>
     </r>
   </si>
   <si>
@@ -983,7 +983,7 @@
       <rPr>
         <family val="2"/>
       </rPr>
-      <t>：落基山脉和大平原影响着天气模式，而密西西比河流域是世界上最肥沃的农业区之一。北美洲还拥有显著的生物多样性，从北极苔原到西南部的沙漠。</t>
+      <t>：落基山脉和大平原影响着天气模式，而密西西比河流域是世界上最肥沃的农业区之一。北美洲还拥有丰富的生物多样性，从北极苔原到西南部的沙漠。</t>
     </r>
   </si>
   <si>
@@ -1007,7 +1007,7 @@
       <rPr>
         <family val="2"/>
       </rPr>
-      <t>：南极冰盖含有全球约70%的淡水。由于气候变化导致的融化可能导致海平面上升，影响全球沿海城市。</t>
+      <t>：南极冰盖含有全球约70%的淡水。气候变化导致的融化可能导致海平面上升，影响全球沿海城市。</t>
     </r>
   </si>
   <si>
@@ -1019,7 +1019,7 @@
       <rPr>
         <family val="2"/>
       </rPr>
-      <t>：欧洲多样化的景观，从阿尔卑斯山到斯堪的纳维亚峡湾，影响着区域气候并支持着丰富的生态系统。该大陆的河流，如多瑙河和莱茵河，对交通和农业至关重要。</t>
+      <t>：欧洲多样化的景观，从阿尔卑斯山到斯堪的纳维亚峡湾，影响着区域气候并支持着丰富的生态系统。欧洲的河流，如多瑙河和莱茵河，对交通和农业至关重要。</t>
     </r>
   </si>
   <si>
@@ -1031,7 +1031,7 @@
       <rPr>
         <family val="2"/>
       </rPr>
-      <t>：澳大利亚独特的生态系统，包括大堡礁和内陆地区，对全球生物多样性做出了贡献。然而，它对气候变化的脆弱性，如丛林大火和珊瑚白化等事件所示，凸显了全球生态系统的相互关联性。</t>
+      <t>：澳大利亚独特的生态系统，包括大堡礁和内陆地区，为全球生物多样性做出了贡献。然而，其对气候变化的脆弱性，如森林大火和珊瑚白化等事件所示，凸显了全球生态系统的相互关联性。</t>
     </r>
   </si>
   <si>
@@ -1049,7 +1049,7 @@
       <rPr>
         <family val="2"/>
       </rPr>
-      <t>：作为主要宗教（印度教、佛教、伊斯兰教和基督教）的发源地，亚洲塑造了全球灵性和哲学。中国和印度等古代文明对科学、数学和文学做出了贡献，影响了世界数千年。</t>
+      <t>：作为主要宗教（印度教、佛教、伊斯兰教和基督教）的发源地，亚洲塑造了全球的灵性和哲学。中国和印度等古代文明对科学、数学和文学做出了贡献，影响了世界数千年。</t>
     </r>
   </si>
   <si>
@@ -1061,7 +1061,7 @@
       <rPr>
         <family val="2"/>
       </rPr>
-      <t>：非洲常被称为“人类摇篮”，是最初人类进化的地方。其丰富的文化遗产，从古埃及到马里帝国，在艺术、建筑和历史上留下了不可磨灭的印记。</t>
+      <t>：非洲常被称为“人类摇篮”，是最初人类的进化之地。其丰富的文化遗产，从古埃及到马里帝国，在艺术、建筑和历史上留下了不可磨灭的印记。</t>
     </r>
   </si>
   <si>
@@ -1073,7 +1073,7 @@
       <rPr>
         <family val="2"/>
       </rPr>
-      <t>：北美洲的土著文化，如纳瓦霍人和易洛魁人，为全球可持续发展和环境管理知识做出了贡献。欧洲殖民和跨大西洋奴隶贸易对全球人口和文化产生了持久影响。</t>
+      <t>：北美洲的土著文化，如纳瓦霍族和易洛魁族，为全球可持续发展和环境管理知识做出了贡献。欧洲殖民和跨大西洋奴隶贸易对全球人口结构和文化产生了持久影响。</t>
     </r>
   </si>
   <si>
@@ -1085,7 +1085,7 @@
       <rPr>
         <family val="2"/>
       </rPr>
-      <t>：印加、玛雅和阿兹特克文明留下了不朽的建筑和先进的农业实践。非洲大陆充满活力的文化，包括音乐、舞蹈和节日，影响了全球艺术和娱乐。</t>
+      <t>：印加、玛雅和阿兹特克文明留下了不朽的建筑和先进的农业实践。该大陆充满活力的文化，包括音乐、舞蹈和节日，影响了全球艺术和娱乐。</t>
     </r>
   </si>
   <si>
@@ -1109,7 +1109,7 @@
       <rPr>
         <family val="2"/>
       </rPr>
-      <t>：拥有超过 65,000 年历史的澳大利亚原住民文化，为可持续生活和与土地的联系提供了深刻的见解。澳大利亚的多元文化社会反映了其作为全球移民中心的地位。</t>
+      <t>：澳大利亚原住民文化拥有超过 65,000 年的历史，为可持续生活和与土地的联系提供了深刻的见解。澳大利亚的多元文化社会反映了其作为全球移民中心的地位。</t>
     </r>
   </si>
   <si>
@@ -1127,7 +1127,7 @@
       <rPr>
         <family val="2"/>
       </rPr>
-      <t>：亚洲是全球经济强国，中国、印度和日本等国家推动着国际贸易和创新。亚洲是电子产品、纺织品和汽车的主要生产国，影响着全球市场。</t>
+      <t>：亚洲是全球经济强国，中国、印度和日本等国家推动着国际贸易和创新。该大陆是电子产品、纺织品和汽车的主要生产商，影响着全球市场。</t>
     </r>
   </si>
   <si>
@@ -1139,7 +1139,7 @@
       <rPr>
         <family val="2"/>
       </rPr>
-      <t>：非洲拥有丰富的自然资源，包括石油、钻石和黄金，这些对全球经济至关重要。然而，贫困和不平等等经济挑战在许多地区依然存在。</t>
+      <t>：非洲拥有丰富的自然资源，包括石油、钻石和黄金，这些对全球经济至关重要。然而，贫困和不平等之类的经济挑战在许多地区依然存在。</t>
     </r>
   </si>
   <si>
@@ -1151,7 +1151,7 @@
       <rPr>
         <family val="2"/>
       </rPr>
-      <t>：美国和加拿大是世界上最大的经济体之一，对技术、金融和娱乐做出了重大贡献。北美洲的农业产出养活了全球数百万人口。</t>
+      <t>：美国和加拿大是世界上最大的经济体之一，对技术、金融和娱乐做出了重大贡献。北美洲的农业产出养活了全球数百万人。</t>
     </r>
   </si>
   <si>
@@ -1163,7 +1163,7 @@
       <rPr>
         <family val="2"/>
       </rPr>
-      <t>：南美洲是大豆、咖啡和铜等商品的主要出口国。巴西是南美洲最大的经济体，在全球贸易中发挥着关键作用。</t>
+      <t>：该大陆是大豆、咖啡和铜等商品的主要出口国。巴西是南美洲最大的经济体，在全球贸易中扮演着关键角色。</t>
     </r>
   </si>
   <si>
@@ -1175,7 +1175,7 @@
       <rPr>
         <family val="2"/>
       </rPr>
-      <t>：欧盟是世界上最大的经济集团之一，促进其成员国之间的贸易与合作。欧洲也是可再生能源和可持续发展的领导者。</t>
+      <t>：欧盟是世界上最大的经济集团之一，促进其成员国之间的贸易和合作。欧洲也是可再生能源和可持续发展的领导者。</t>
     </r>
   </si>
   <si>
@@ -1205,7 +1205,7 @@
       <rPr>
         <family val="2"/>
       </rPr>
-      <t>：亚洲的地缘政治意义不可否认，中国、印度和日本等国家在国际关系中发挥着关键作用。该地区的冲突和联盟塑造了全球政治。</t>
+      <t>：亚洲的地缘政治意义不可否认，中国、印度和日本等国家在国际关系中扮演着关键角色。该地区的冲突和联盟影响着全球政治。</t>
     </r>
   </si>
   <si>
@@ -1217,7 +1217,7 @@
       <rPr>
         <family val="2"/>
       </rPr>
-      <t>：非洲不断增长的人口和年轻的人口结构使其成为全球发展中的关键参与者。非洲大陆为应对贫困、健康危机和政治不稳定等挑战所做的努力具有深远影响。</t>
+      <t>：非洲不断增长的人口和年轻的人口结构使其成为全球发展中的关键参与者。该大陆应对贫困、健康危机和政治不稳定等挑战的努力具有深远的影响。</t>
     </r>
   </si>
   <si>
@@ -1241,7 +1241,7 @@
       <rPr>
         <family val="2"/>
       </rPr>
-      <t>：南美洲的政治格局，从委内瑞拉的社会主义运动到智利的民主转型，反映了其多元的意识形态和争取平等的斗争。</t>
+      <t>：该大陆的政治格局，从委内瑞拉的社会主义运动到智利的民主转型，反映了其多元的意识形态和对平等的斗争。</t>
     </r>
   </si>
   <si>
@@ -1265,7 +1265,7 @@
       <rPr>
         <family val="2"/>
       </rPr>
-      <t>：澳大利亚在亚太地区的作用以及其对国际援助和环境保护的承诺，凸显了其全球影响力。</t>
+      <t>：澳大利亚在亚太地区的作用及其对国际援助和环境保护的承诺突显了其全球影响力。</t>
     </r>
   </si>
   <si>
@@ -1313,7 +1313,7 @@
       <rPr>
         <family val="2"/>
       </rPr>
-      <t>：经历野火、飓风和北极冰融化。</t>
+      <t>：经历森林火灾、飓风和北极冰融化。</t>
     </r>
   </si>
   <si>
@@ -1349,7 +1349,7 @@
       <rPr>
         <family val="2"/>
       </rPr>
-      <t>：面临气候变化导致的酷热和洪水。</t>
+      <t>：面临气候变化导致的热浪和洪水。</t>
     </r>
   </si>
   <si>
@@ -1373,7 +1373,7 @@
   <si>
     <r>
       <rPr/>
-      <t>各大洲通过贸易、移民和技术相互关联。例如：</t>
+      <t>各大洲通过贸易、移民和技术相互连接。例如：</t>
     </r>
   </si>
   <si>
@@ -1397,7 +1397,7 @@
       <rPr>
         <family val="2"/>
       </rPr>
-      <t>：人们为了工作、教育和寻求庇护而在各大洲之间迁移，丰富了文化和经济。</t>
+      <t>：人们为了工作、教育和寻求庇护而在各大洲之间迁徙，丰富了文化和经济。</t>
     </r>
   </si>
   <si>
@@ -1415,7 +1415,7 @@
   <si>
     <r>
       <rPr/>
-      <t>世界各大洲并非孤立的实体，而是全球体系中相互关联的部分。它们在地理、文化、经济和政治方面的影响深刻地塑造着世界。面对气候变化、不平等和冲突等全球性挑战，了解各大洲的作用和贡献对于促进合作、为全人类创造可持续的未来至关重要。通过认识到各大洲的多样性和相互关联性，我们可以共同努力应对共同挑战，建设一个更美好的世界。</t>
+      <t>世界各大洲并非孤立的实体，而是全球系统中相互关联的部分。它们的地理、文化、经济和政治影响深刻地塑造着世界。当我们面临气候变化、不平等和冲突等全球性挑战时，了解每个大洲的作用和贡献对于促进合作、为所有人创造可持续的未来至关重要。通过认识到各大洲的多样性和相互关联性，我们可以共同努力应对共同挑战，建设一个更美好的世界。</t>
     </r>
   </si>
 </sst>

</xml_diff>